<commit_message>
updated whatsapp blaster code
</commit_message>
<xml_diff>
--- a/scripts/eauto-insurance/input-vehicles.xlsx
+++ b/scripts/eauto-insurance/input-vehicles.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,10 +415,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BHA2468</v>
+        <v>WKR590</v>
       </c>
       <c r="B2" t="str">
-        <v>030303-A</v>
+        <v>030217141005</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -429,10 +429,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CCF5361</v>
+        <v>MU1977</v>
       </c>
       <c r="B3" t="str">
-        <v>030303-A</v>
+        <v>030217141005</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -443,10 +443,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>QAB3377M</v>
+        <v>QAA8160F</v>
       </c>
       <c r="B4" t="str">
-        <v>030303-A</v>
+        <v>030217141005</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -457,63 +457,21 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>VDA9008</v>
+        <v>WWK7705</v>
       </c>
       <c r="B5" t="str">
-        <v>030303-A</v>
+        <v>030217141005</v>
       </c>
       <c r="C5" t="str">
         <v/>
       </c>
       <c r="D5" t="str">
-        <v>company</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>WYX8315</v>
-      </c>
-      <c r="B6" t="str">
-        <v>030303-A</v>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v>company</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>WVY6520</v>
-      </c>
-      <c r="B7" t="str">
-        <v>030303-A</v>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v>company</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>WVY6520</v>
-      </c>
-      <c r="B8" t="str">
-        <v>030303-A</v>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
         <v>company</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Latest update on all automation script
</commit_message>
<xml_diff>
--- a/scripts/eauto-insurance/input-vehicles.xlsx
+++ b/scripts/eauto-insurance/input-vehicles.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,7 +415,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>JVK1779</v>
+        <v>VPM7358</v>
       </c>
       <c r="B2" t="str">
         <v>030217141005</v>
@@ -424,264 +424,12 @@
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>PRR5421</v>
-      </c>
-      <c r="B3" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>WB7932R</v>
-      </c>
-      <c r="B4" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>WTX9642</v>
-      </c>
-      <c r="B5" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>WEN7866</v>
-      </c>
-      <c r="B6" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>MCH2151</v>
-      </c>
-      <c r="B7" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>WTX9642</v>
-      </c>
-      <c r="B8" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>VMM949</v>
-      </c>
-      <c r="B9" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>JSS9468</v>
-      </c>
-      <c r="B10" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>RW3512</v>
-      </c>
-      <c r="B11" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>BKN9186</v>
-      </c>
-      <c r="B12" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C12" t="str">
-        <v/>
-      </c>
-      <c r="D12" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>JLY4743</v>
-      </c>
-      <c r="B13" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C13" t="str">
-        <v/>
-      </c>
-      <c r="D13" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>VBY8385</v>
-      </c>
-      <c r="B14" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>JPK5366</v>
-      </c>
-      <c r="B15" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>JGC7679</v>
-      </c>
-      <c r="B16" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>JLY4743</v>
-      </c>
-      <c r="B17" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>VPF1134</v>
-      </c>
-      <c r="B18" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>VCK772</v>
-      </c>
-      <c r="B19" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str">
-        <v>individual</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>VDS5747</v>
-      </c>
-      <c r="B20" t="str">
-        <v>030217141005</v>
-      </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
-      <c r="D20" t="str">
         <v>individual</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>